<commit_message>
LotR game posters added and Percy Jackson books added
</commit_message>
<xml_diff>
--- a/MIDDLEEARTH.xlsx
+++ b/MIDDLEEARTH.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348B975D-3248-4B7E-89C3-B644A82B1652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F0C0C89-F21F-4732-867F-D17C06C6B474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="257">
   <si>
     <t>id</t>
   </si>
@@ -64,9 +64,6 @@
     <t>tmdb id</t>
   </si>
   <si>
-    <t>tmdb type</t>
-  </si>
-  <si>
     <t>library url</t>
   </si>
   <si>
@@ -145,9 +142,6 @@
     <t>https://www.themoviedb.org/tv/84773-the-lord-of-the-rings-the-rings-of-power/season/1</t>
   </si>
   <si>
-    <t>tv</t>
-  </si>
-  <si>
     <t>MIDDLEEARTH-0025</t>
   </si>
   <si>
@@ -433,9 +427,6 @@
     <t>https://www.themoviedb.org/movie/839033-the-lord-of-the-rings-the-war-of-the-rohirrim</t>
   </si>
   <si>
-    <t>movie</t>
-  </si>
-  <si>
     <t>MIDDLEEARTH-0001</t>
   </si>
   <si>
@@ -749,6 +740,57 @@
   </si>
   <si>
     <t>https://covers.openlibrary.org/b/id/15246805-L.jpg</t>
+  </si>
+  <si>
+    <t>igdb url</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/tales-of-the-shire</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_big_x2/co84g9.webp</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/middle-earth-shadow-of-mordor</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/middle-earth-shadow-of-war</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/the-lord-of-the-rings-gollum</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/the-lord-of-the-rings-the-battle-for-middle-earth</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/the-lord-of-the-rings-the-battle-for-middle-earth-ii</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/the-lord-of-the-rings-war-in-the-north</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/the-lord-of-the-rings-return-to-moria#media</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_bix_x2/co20pd.webp</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_bix_x2/co20pq.webp</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_bix_x2/co4sdl.webp</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_bix_x2/co20og.webp</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_bix_x2/co20oh.webp</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_bix_x2/co20p9.webp</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_bix_x2/co7a7g.webp</t>
   </si>
 </sst>
 </file>
@@ -1133,19 +1175,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P53"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.3984375" customWidth="1"/>
-    <col min="4" max="4" width="67.73046875" customWidth="1"/>
-    <col min="6" max="6" width="25.86328125" customWidth="1"/>
-    <col min="7" max="7" width="17.86328125" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="4" max="4" width="67.7109375" customWidth="1"/>
+    <col min="6" max="6" width="25.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="50.265625" customWidth="1"/>
-    <col min="12" max="12" width="72.265625" customWidth="1"/>
-    <col min="13" max="13" width="51.1328125" customWidth="1"/>
+    <col min="11" max="11" width="50.28515625" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" customWidth="1"/>
+    <col min="13" max="13" width="18.5703125" customWidth="1"/>
+    <col min="14" max="14" width="20.85546875" customWidth="1"/>
+    <col min="15" max="15" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1192,12 +1236,12 @@
         <v>14</v>
       </c>
       <c r="P1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>16</v>
       </c>
       <c r="B2">
         <v>5</v>
@@ -1206,27 +1250,27 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G2" s="1">
         <v>28383</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="O2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="P2" t="s">
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>21</v>
       </c>
       <c r="B3">
         <v>15</v>
@@ -1235,27 +1279,27 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G3" s="1">
         <v>39189</v>
       </c>
       <c r="I3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K3" t="s">
-        <v>235</v>
-      </c>
-      <c r="P3" t="s">
+        <v>232</v>
+      </c>
+      <c r="O3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>24</v>
       </c>
       <c r="B4">
         <v>21</v>
@@ -1264,27 +1308,27 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G4" s="1">
         <v>42887</v>
       </c>
       <c r="I4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K4" t="s">
-        <v>236</v>
-      </c>
-      <c r="P4" t="s">
+        <v>233</v>
+      </c>
+      <c r="O4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>27</v>
       </c>
       <c r="B5">
         <v>23</v>
@@ -1293,27 +1337,27 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G5" s="1">
         <v>43342</v>
       </c>
       <c r="I5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K5" t="s">
-        <v>237</v>
-      </c>
-      <c r="P5" t="s">
+        <v>234</v>
+      </c>
+      <c r="O5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>30</v>
       </c>
       <c r="B6">
         <v>9</v>
@@ -1322,27 +1366,27 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G6" s="1">
         <v>29496</v>
       </c>
       <c r="I6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K6" t="s">
-        <v>238</v>
-      </c>
-      <c r="P6" t="s">
+        <v>235</v>
+      </c>
+      <c r="O6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>33</v>
       </c>
       <c r="B7">
         <v>24</v>
@@ -1351,13 +1395,13 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
         <v>34</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>35</v>
-      </c>
-      <c r="F7" t="s">
-        <v>36</v>
       </c>
       <c r="G7" s="1">
         <v>44804</v>
@@ -1366,27 +1410,24 @@
         <v>65</v>
       </c>
       <c r="I7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" t="s">
         <v>37</v>
       </c>
-      <c r="J7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="M7" t="s">
         <v>38</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>39</v>
       </c>
-      <c r="N7" t="s">
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>40</v>
-      </c>
-      <c r="O7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>42</v>
       </c>
       <c r="B8">
         <v>25</v>
@@ -1395,13 +1436,13 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G8" s="1">
         <v>44804</v>
@@ -1410,27 +1451,24 @@
         <v>67</v>
       </c>
       <c r="I8" t="s">
+        <v>36</v>
+      </c>
+      <c r="J8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K8" t="s">
         <v>37</v>
       </c>
-      <c r="J8" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" t="s">
-        <v>38</v>
-      </c>
       <c r="M8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N8" t="s">
-        <v>40</v>
-      </c>
-      <c r="O8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B9">
         <v>26</v>
@@ -1439,13 +1477,13 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G9" s="1">
         <v>44812</v>
@@ -1454,27 +1492,24 @@
         <v>69</v>
       </c>
       <c r="I9" t="s">
+        <v>36</v>
+      </c>
+      <c r="J9" t="s">
+        <v>18</v>
+      </c>
+      <c r="K9" t="s">
         <v>37</v>
       </c>
-      <c r="J9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" t="s">
-        <v>38</v>
-      </c>
       <c r="M9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="N9" t="s">
-        <v>40</v>
-      </c>
-      <c r="O9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B10">
         <v>27</v>
@@ -1483,13 +1518,13 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G10" s="1">
         <v>44819</v>
@@ -1498,27 +1533,24 @@
         <v>71</v>
       </c>
       <c r="I10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J10" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" t="s">
         <v>37</v>
       </c>
-      <c r="J10" t="s">
-        <v>19</v>
-      </c>
-      <c r="K10" t="s">
-        <v>38</v>
-      </c>
       <c r="M10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="N10" t="s">
-        <v>40</v>
-      </c>
-      <c r="O10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B11">
         <v>28</v>
@@ -1527,13 +1559,13 @@
         <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G11" s="1">
         <v>44826</v>
@@ -1542,27 +1574,24 @@
         <v>72</v>
       </c>
       <c r="I11" t="s">
+        <v>36</v>
+      </c>
+      <c r="J11" t="s">
+        <v>18</v>
+      </c>
+      <c r="K11" t="s">
         <v>37</v>
       </c>
-      <c r="J11" t="s">
-        <v>19</v>
-      </c>
-      <c r="K11" t="s">
-        <v>38</v>
-      </c>
       <c r="M11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N11" t="s">
-        <v>40</v>
-      </c>
-      <c r="O11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B12">
         <v>29</v>
@@ -1571,13 +1600,13 @@
         <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G12" s="1">
         <v>44833</v>
@@ -1586,27 +1615,24 @@
         <v>69</v>
       </c>
       <c r="I12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J12" t="s">
+        <v>18</v>
+      </c>
+      <c r="K12" t="s">
         <v>37</v>
       </c>
-      <c r="J12" t="s">
-        <v>19</v>
-      </c>
-      <c r="K12" t="s">
-        <v>38</v>
-      </c>
       <c r="M12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N12" t="s">
-        <v>40</v>
-      </c>
-      <c r="O12" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B13">
         <v>30</v>
@@ -1615,13 +1641,13 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G13" s="1">
         <v>44840</v>
@@ -1630,27 +1656,24 @@
         <v>72</v>
       </c>
       <c r="I13" t="s">
+        <v>36</v>
+      </c>
+      <c r="J13" t="s">
+        <v>18</v>
+      </c>
+      <c r="K13" t="s">
         <v>37</v>
       </c>
-      <c r="J13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" t="s">
-        <v>38</v>
-      </c>
       <c r="M13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="N13" t="s">
-        <v>40</v>
-      </c>
-      <c r="O13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B14">
         <v>31</v>
@@ -1659,13 +1682,13 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G14" s="1">
         <v>44847</v>
@@ -1674,27 +1697,24 @@
         <v>72</v>
       </c>
       <c r="I14" t="s">
+        <v>36</v>
+      </c>
+      <c r="J14" t="s">
+        <v>18</v>
+      </c>
+      <c r="K14" t="s">
         <v>37</v>
       </c>
-      <c r="J14" t="s">
-        <v>19</v>
-      </c>
-      <c r="K14" t="s">
-        <v>38</v>
-      </c>
       <c r="M14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N14" t="s">
-        <v>40</v>
-      </c>
-      <c r="O14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B15">
         <v>34</v>
@@ -1703,13 +1723,13 @@
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G15" s="1">
         <v>45532</v>
@@ -1718,27 +1738,24 @@
         <v>76</v>
       </c>
       <c r="I15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K15" t="s">
+        <v>71</v>
+      </c>
+      <c r="M15" t="s">
+        <v>72</v>
+      </c>
+      <c r="N15" t="s">
         <v>73</v>
       </c>
-      <c r="M15" t="s">
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>74</v>
-      </c>
-      <c r="N15" t="s">
-        <v>75</v>
-      </c>
-      <c r="O15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>76</v>
       </c>
       <c r="B16">
         <v>35</v>
@@ -1747,13 +1764,13 @@
         <v>15</v>
       </c>
       <c r="D16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E16" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G16" s="1">
         <v>45532</v>
@@ -1762,27 +1779,24 @@
         <v>62</v>
       </c>
       <c r="I16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K16" t="s">
+        <v>71</v>
+      </c>
+      <c r="M16" t="s">
+        <v>77</v>
+      </c>
+      <c r="N16" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="M16" t="s">
-        <v>79</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="O16" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B17">
         <v>36</v>
@@ -1791,13 +1805,13 @@
         <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G17" s="1">
         <v>45532</v>
@@ -1806,27 +1820,24 @@
         <v>66</v>
       </c>
       <c r="I17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K17" t="s">
+        <v>71</v>
+      </c>
+      <c r="M17" t="s">
+        <v>81</v>
+      </c>
+      <c r="N17" t="s">
         <v>73</v>
       </c>
-      <c r="M17" t="s">
-        <v>83</v>
-      </c>
-      <c r="N17" t="s">
-        <v>75</v>
-      </c>
-      <c r="O17" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B18">
         <v>37</v>
@@ -1835,13 +1846,13 @@
         <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F18" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G18" s="1">
         <v>45539</v>
@@ -1850,27 +1861,24 @@
         <v>65</v>
       </c>
       <c r="I18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K18" t="s">
+        <v>71</v>
+      </c>
+      <c r="M18" t="s">
+        <v>85</v>
+      </c>
+      <c r="N18" t="s">
         <v>73</v>
       </c>
-      <c r="M18" t="s">
-        <v>87</v>
-      </c>
-      <c r="N18" t="s">
-        <v>75</v>
-      </c>
-      <c r="O18" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B19">
         <v>38</v>
@@ -1879,13 +1887,13 @@
         <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E19" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G19" s="1">
         <v>45546</v>
@@ -1894,27 +1902,24 @@
         <v>61</v>
       </c>
       <c r="I19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K19" t="s">
+        <v>71</v>
+      </c>
+      <c r="M19" t="s">
+        <v>89</v>
+      </c>
+      <c r="N19" t="s">
         <v>73</v>
       </c>
-      <c r="M19" t="s">
-        <v>91</v>
-      </c>
-      <c r="N19" t="s">
-        <v>75</v>
-      </c>
-      <c r="O19" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B20">
         <v>39</v>
@@ -1923,13 +1928,13 @@
         <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F20" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G20" s="1">
         <v>45553</v>
@@ -1938,27 +1943,24 @@
         <v>63</v>
       </c>
       <c r="I20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K20" t="s">
+        <v>71</v>
+      </c>
+      <c r="M20" t="s">
+        <v>93</v>
+      </c>
+      <c r="N20" t="s">
         <v>73</v>
       </c>
-      <c r="M20" t="s">
-        <v>95</v>
-      </c>
-      <c r="N20" t="s">
-        <v>75</v>
-      </c>
-      <c r="O20" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B21">
         <v>40</v>
@@ -1967,13 +1969,13 @@
         <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E21" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F21" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G21" s="1">
         <v>45560</v>
@@ -1982,27 +1984,24 @@
         <v>72</v>
       </c>
       <c r="I21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K21" t="s">
+        <v>71</v>
+      </c>
+      <c r="M21" t="s">
+        <v>97</v>
+      </c>
+      <c r="N21" t="s">
         <v>73</v>
       </c>
-      <c r="M21" t="s">
-        <v>99</v>
-      </c>
-      <c r="N21" t="s">
-        <v>75</v>
-      </c>
-      <c r="O21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B22">
         <v>41</v>
@@ -2011,13 +2010,13 @@
         <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E22" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G22" s="1">
         <v>45567</v>
@@ -2026,27 +2025,24 @@
         <v>73</v>
       </c>
       <c r="I22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K22" t="s">
+        <v>71</v>
+      </c>
+      <c r="M22" t="s">
+        <v>101</v>
+      </c>
+      <c r="N22" t="s">
         <v>73</v>
       </c>
-      <c r="M22" t="s">
-        <v>103</v>
-      </c>
-      <c r="N22" t="s">
-        <v>75</v>
-      </c>
-      <c r="O22" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B23">
         <v>44</v>
@@ -2055,36 +2051,33 @@
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E23" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G23" s="1">
         <v>46337</v>
       </c>
       <c r="I23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K23" t="s">
+        <v>104</v>
+      </c>
+      <c r="M23" t="s">
+        <v>105</v>
+      </c>
+      <c r="N23" t="s">
         <v>106</v>
       </c>
-      <c r="M23" t="s">
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>107</v>
-      </c>
-      <c r="N23" t="s">
-        <v>108</v>
-      </c>
-      <c r="O23" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>109</v>
       </c>
       <c r="B24">
         <v>45</v>
@@ -2093,36 +2086,33 @@
         <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E24" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G24" s="1">
         <v>46337</v>
       </c>
       <c r="I24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K24" t="s">
+        <v>104</v>
+      </c>
+      <c r="M24" t="s">
+        <v>109</v>
+      </c>
+      <c r="N24" t="s">
         <v>106</v>
       </c>
-      <c r="M24" t="s">
-        <v>111</v>
-      </c>
-      <c r="N24" t="s">
-        <v>108</v>
-      </c>
-      <c r="O24" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B25">
         <v>46</v>
@@ -2131,36 +2121,33 @@
         <v>24</v>
       </c>
       <c r="D25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E25" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G25" s="1">
         <v>46337</v>
       </c>
       <c r="I25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K25" t="s">
+        <v>104</v>
+      </c>
+      <c r="M25" t="s">
+        <v>112</v>
+      </c>
+      <c r="N25" t="s">
         <v>106</v>
       </c>
-      <c r="M25" t="s">
-        <v>114</v>
-      </c>
-      <c r="N25" t="s">
-        <v>108</v>
-      </c>
-      <c r="O25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B26">
         <v>47</v>
@@ -2169,36 +2156,33 @@
         <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E26" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G26" s="1">
         <v>46337</v>
       </c>
       <c r="I26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K26" t="s">
+        <v>104</v>
+      </c>
+      <c r="M26" t="s">
+        <v>115</v>
+      </c>
+      <c r="N26" t="s">
         <v>106</v>
       </c>
-      <c r="M26" t="s">
-        <v>117</v>
-      </c>
-      <c r="N26" t="s">
-        <v>108</v>
-      </c>
-      <c r="O26" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B27">
         <v>48</v>
@@ -2207,36 +2191,33 @@
         <v>26</v>
       </c>
       <c r="D27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G27" s="1">
         <v>46344</v>
       </c>
       <c r="I27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K27" t="s">
+        <v>104</v>
+      </c>
+      <c r="M27" t="s">
+        <v>118</v>
+      </c>
+      <c r="N27" t="s">
         <v>106</v>
       </c>
-      <c r="M27" t="s">
-        <v>120</v>
-      </c>
-      <c r="N27" t="s">
-        <v>108</v>
-      </c>
-      <c r="O27" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B28">
         <v>49</v>
@@ -2245,36 +2226,33 @@
         <v>27</v>
       </c>
       <c r="D28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G28" s="1">
         <v>46344</v>
       </c>
       <c r="I28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K28" t="s">
+        <v>104</v>
+      </c>
+      <c r="M28" t="s">
+        <v>121</v>
+      </c>
+      <c r="N28" t="s">
         <v>106</v>
       </c>
-      <c r="M28" t="s">
-        <v>123</v>
-      </c>
-      <c r="N28" t="s">
-        <v>108</v>
-      </c>
-      <c r="O28" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B29">
         <v>50</v>
@@ -2283,36 +2261,33 @@
         <v>28</v>
       </c>
       <c r="D29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E29" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G29" s="1">
         <v>46351</v>
       </c>
       <c r="I29" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K29" t="s">
+        <v>104</v>
+      </c>
+      <c r="M29" t="s">
+        <v>124</v>
+      </c>
+      <c r="N29" t="s">
         <v>106</v>
       </c>
-      <c r="M29" t="s">
-        <v>126</v>
-      </c>
-      <c r="N29" t="s">
-        <v>108</v>
-      </c>
-      <c r="O29" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B30">
         <v>51</v>
@@ -2321,36 +2296,33 @@
         <v>29</v>
       </c>
       <c r="D30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E30" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G30" s="1">
         <v>46351</v>
       </c>
       <c r="I30" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J30" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K30" t="s">
+        <v>104</v>
+      </c>
+      <c r="M30" t="s">
+        <v>127</v>
+      </c>
+      <c r="N30" t="s">
         <v>106</v>
       </c>
-      <c r="M30" t="s">
-        <v>129</v>
-      </c>
-      <c r="N30" t="s">
-        <v>108</v>
-      </c>
-      <c r="O30" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.45">
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B31">
         <v>42</v>
@@ -2359,7 +2331,7 @@
         <v>30</v>
       </c>
       <c r="D31" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G31" s="1">
         <v>45639</v>
@@ -2368,30 +2340,27 @@
         <v>134</v>
       </c>
       <c r="I31" t="s">
+        <v>130</v>
+      </c>
+      <c r="J31" t="s">
+        <v>18</v>
+      </c>
+      <c r="K31" t="s">
+        <v>131</v>
+      </c>
+      <c r="L31" t="s">
         <v>132</v>
       </c>
-      <c r="J31" t="s">
-        <v>19</v>
-      </c>
-      <c r="K31" t="s">
+      <c r="M31" t="s">
         <v>133</v>
       </c>
-      <c r="L31" t="s">
+      <c r="N31" t="s">
         <v>134</v>
       </c>
-      <c r="M31" t="s">
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>135</v>
-      </c>
-      <c r="N31" t="s">
-        <v>136</v>
-      </c>
-      <c r="O31" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
-        <v>138</v>
       </c>
       <c r="B32">
         <v>1</v>
@@ -2400,27 +2369,27 @@
         <v>31</v>
       </c>
       <c r="D32" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G32" s="1">
         <v>13779</v>
       </c>
       <c r="I32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J32" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K32" t="s">
-        <v>239</v>
-      </c>
-      <c r="P32" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.45">
+        <v>236</v>
+      </c>
+      <c r="O32" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B33">
         <v>6</v>
@@ -2429,7 +2398,7 @@
         <v>32</v>
       </c>
       <c r="D33" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G33" s="1">
         <v>28456</v>
@@ -2438,30 +2407,27 @@
         <v>78</v>
       </c>
       <c r="I33" t="s">
+        <v>139</v>
+      </c>
+      <c r="J33" t="s">
+        <v>18</v>
+      </c>
+      <c r="K33" t="s">
+        <v>140</v>
+      </c>
+      <c r="L33" t="s">
+        <v>141</v>
+      </c>
+      <c r="M33" t="s">
         <v>142</v>
       </c>
-      <c r="J33" t="s">
-        <v>19</v>
-      </c>
-      <c r="K33" t="s">
+      <c r="N33" t="s">
         <v>143</v>
       </c>
-      <c r="L33" t="s">
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>144</v>
-      </c>
-      <c r="M33" t="s">
-        <v>145</v>
-      </c>
-      <c r="N33" t="s">
-        <v>146</v>
-      </c>
-      <c r="O33" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
-        <v>147</v>
       </c>
       <c r="B34">
         <v>17</v>
@@ -2470,7 +2436,7 @@
         <v>33</v>
       </c>
       <c r="D34" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G34" s="1">
         <v>41257</v>
@@ -2479,30 +2445,27 @@
         <v>182</v>
       </c>
       <c r="I34" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J34" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K34" t="s">
+        <v>146</v>
+      </c>
+      <c r="L34" t="s">
+        <v>147</v>
+      </c>
+      <c r="M34" t="s">
+        <v>148</v>
+      </c>
+      <c r="N34" t="s">
         <v>149</v>
       </c>
-      <c r="L34" t="s">
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>150</v>
-      </c>
-      <c r="M34" t="s">
-        <v>151</v>
-      </c>
-      <c r="N34" t="s">
-        <v>152</v>
-      </c>
-      <c r="O34" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
-        <v>153</v>
       </c>
       <c r="B35">
         <v>18</v>
@@ -2511,7 +2474,7 @@
         <v>34</v>
       </c>
       <c r="D35" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="G35" s="1">
         <v>41621</v>
@@ -2520,30 +2483,27 @@
         <v>186</v>
       </c>
       <c r="I35" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K35" t="s">
+        <v>152</v>
+      </c>
+      <c r="L35" t="s">
+        <v>153</v>
+      </c>
+      <c r="M35" t="s">
+        <v>154</v>
+      </c>
+      <c r="N35" t="s">
         <v>155</v>
       </c>
-      <c r="L35" t="s">
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>156</v>
-      </c>
-      <c r="M35" t="s">
-        <v>157</v>
-      </c>
-      <c r="N35" t="s">
-        <v>158</v>
-      </c>
-      <c r="O35" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
-        <v>159</v>
       </c>
       <c r="B36">
         <v>20</v>
@@ -2552,7 +2512,7 @@
         <v>35</v>
       </c>
       <c r="D36" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G36" s="1">
         <v>41990</v>
@@ -2561,30 +2521,27 @@
         <v>164</v>
       </c>
       <c r="I36" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K36" t="s">
+        <v>158</v>
+      </c>
+      <c r="L36" t="s">
+        <v>159</v>
+      </c>
+      <c r="M36" t="s">
+        <v>160</v>
+      </c>
+      <c r="N36" t="s">
         <v>161</v>
       </c>
-      <c r="L36" t="s">
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>162</v>
-      </c>
-      <c r="M36" t="s">
-        <v>163</v>
-      </c>
-      <c r="N36" t="s">
-        <v>164</v>
-      </c>
-      <c r="O36" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
-        <v>165</v>
       </c>
       <c r="B37">
         <v>43</v>
@@ -2593,24 +2550,30 @@
         <v>36</v>
       </c>
       <c r="D37" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G37" s="1">
         <v>45867</v>
       </c>
       <c r="I37" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J37" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>242</v>
       </c>
       <c r="M37" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.45">
+        <v>165</v>
+      </c>
+      <c r="P37" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B38">
         <v>19</v>
@@ -2619,24 +2582,30 @@
         <v>37</v>
       </c>
       <c r="D38" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="G38" s="1">
         <v>41912</v>
       </c>
       <c r="I38" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J38" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="K38" t="s">
+        <v>250</v>
       </c>
       <c r="M38" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.45">
+        <v>168</v>
+      </c>
+      <c r="P38" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B39">
         <v>22</v>
@@ -2645,24 +2614,30 @@
         <v>38</v>
       </c>
       <c r="D39" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="G39" s="1">
         <v>43018</v>
       </c>
       <c r="I39" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J39" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="K39" t="s">
+        <v>251</v>
       </c>
       <c r="M39" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.45">
+        <v>171</v>
+      </c>
+      <c r="P39" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B40">
         <v>32</v>
@@ -2671,24 +2646,30 @@
         <v>39</v>
       </c>
       <c r="D40" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="G40" s="1">
         <v>45071</v>
       </c>
       <c r="I40" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J40" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="K40" t="s">
+        <v>252</v>
       </c>
       <c r="M40" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.45">
+        <v>174</v>
+      </c>
+      <c r="P40" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B41">
         <v>52</v>
@@ -2697,36 +2678,33 @@
         <v>40</v>
       </c>
       <c r="D41" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G41" s="1">
         <v>46738</v>
       </c>
       <c r="I41" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J41" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K41" t="s">
+        <v>177</v>
+      </c>
+      <c r="L41" t="s">
+        <v>178</v>
+      </c>
+      <c r="M41" t="s">
+        <v>179</v>
+      </c>
+      <c r="N41" t="s">
         <v>180</v>
       </c>
-      <c r="L41" t="s">
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>181</v>
-      </c>
-      <c r="M41" t="s">
-        <v>182</v>
-      </c>
-      <c r="N41" t="s">
-        <v>183</v>
-      </c>
-      <c r="O41" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
-        <v>184</v>
       </c>
       <c r="B42">
         <v>2</v>
@@ -2735,27 +2713,27 @@
         <v>41</v>
       </c>
       <c r="D42" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="G42" s="1">
         <v>19934</v>
       </c>
       <c r="I42" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J42" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K42" t="s">
-        <v>240</v>
-      </c>
-      <c r="P42" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.45">
+        <v>237</v>
+      </c>
+      <c r="O42" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B43">
         <v>10</v>
@@ -2764,7 +2742,7 @@
         <v>42</v>
       </c>
       <c r="D43" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="G43" s="1">
         <v>37244</v>
@@ -2773,30 +2751,27 @@
         <v>228</v>
       </c>
       <c r="I43" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J43" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K43" t="s">
+        <v>186</v>
+      </c>
+      <c r="L43" t="s">
+        <v>187</v>
+      </c>
+      <c r="M43" t="s">
+        <v>188</v>
+      </c>
+      <c r="N43" t="s">
         <v>189</v>
       </c>
-      <c r="L43" t="s">
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>190</v>
-      </c>
-      <c r="M43" t="s">
-        <v>191</v>
-      </c>
-      <c r="N43" t="s">
-        <v>192</v>
-      </c>
-      <c r="O43" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A44" t="s">
-        <v>193</v>
       </c>
       <c r="B44">
         <v>3</v>
@@ -2805,27 +2780,27 @@
         <v>43</v>
       </c>
       <c r="D44" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G44" s="1">
         <v>20039</v>
       </c>
       <c r="I44" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J44" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K44" t="s">
-        <v>241</v>
-      </c>
-      <c r="P44" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.45">
+        <v>238</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B45">
         <v>7</v>
@@ -2834,7 +2809,7 @@
         <v>44</v>
       </c>
       <c r="D45" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="G45" s="1">
         <v>28809</v>
@@ -2843,30 +2818,27 @@
         <v>132</v>
       </c>
       <c r="I45" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="J45" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K45" t="s">
+        <v>195</v>
+      </c>
+      <c r="L45" t="s">
+        <v>196</v>
+      </c>
+      <c r="M45" t="s">
+        <v>197</v>
+      </c>
+      <c r="N45" t="s">
         <v>198</v>
       </c>
-      <c r="L45" t="s">
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>199</v>
-      </c>
-      <c r="M45" t="s">
-        <v>200</v>
-      </c>
-      <c r="N45" t="s">
-        <v>201</v>
-      </c>
-      <c r="O45" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A46" t="s">
-        <v>202</v>
       </c>
       <c r="B46">
         <v>11</v>
@@ -2875,7 +2847,7 @@
         <v>45</v>
       </c>
       <c r="D46" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="G46" s="1">
         <v>37608</v>
@@ -2884,30 +2856,27 @@
         <v>235</v>
       </c>
       <c r="I46" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J46" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K46" t="s">
+        <v>201</v>
+      </c>
+      <c r="L46" t="s">
+        <v>202</v>
+      </c>
+      <c r="M46" t="s">
+        <v>203</v>
+      </c>
+      <c r="N46" t="s">
         <v>204</v>
       </c>
-      <c r="L46" t="s">
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>205</v>
-      </c>
-      <c r="M46" t="s">
-        <v>206</v>
-      </c>
-      <c r="N46" t="s">
-        <v>207</v>
-      </c>
-      <c r="O46" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A47" t="s">
-        <v>208</v>
       </c>
       <c r="B47">
         <v>4</v>
@@ -2916,27 +2885,27 @@
         <v>46</v>
       </c>
       <c r="D47" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G47" s="1">
         <v>20382</v>
       </c>
       <c r="I47" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J47" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K47" t="s">
-        <v>242</v>
-      </c>
-      <c r="P47" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.45">
+        <v>239</v>
+      </c>
+      <c r="O47" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B48">
         <v>8</v>
@@ -2945,7 +2914,7 @@
         <v>47</v>
       </c>
       <c r="D48" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G48" s="1">
         <v>29352</v>
@@ -2954,30 +2923,27 @@
         <v>98</v>
       </c>
       <c r="I48" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="J48" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K48" t="s">
+        <v>209</v>
+      </c>
+      <c r="L48" t="s">
+        <v>210</v>
+      </c>
+      <c r="M48" t="s">
+        <v>211</v>
+      </c>
+      <c r="N48" t="s">
         <v>212</v>
       </c>
-      <c r="L48" t="s">
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>213</v>
-      </c>
-      <c r="M48" t="s">
-        <v>214</v>
-      </c>
-      <c r="N48" t="s">
-        <v>215</v>
-      </c>
-      <c r="O48" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A49" t="s">
-        <v>216</v>
       </c>
       <c r="B49">
         <v>12</v>
@@ -2986,7 +2952,7 @@
         <v>48</v>
       </c>
       <c r="D49" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="G49" s="1">
         <v>37972</v>
@@ -2995,30 +2961,27 @@
         <v>263</v>
       </c>
       <c r="I49" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J49" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K49" t="s">
+        <v>215</v>
+      </c>
+      <c r="L49" t="s">
+        <v>216</v>
+      </c>
+      <c r="M49" t="s">
+        <v>217</v>
+      </c>
+      <c r="N49" t="s">
         <v>218</v>
       </c>
-      <c r="L49" t="s">
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>219</v>
-      </c>
-      <c r="M49" t="s">
-        <v>220</v>
-      </c>
-      <c r="N49" t="s">
-        <v>221</v>
-      </c>
-      <c r="O49" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A50" t="s">
-        <v>222</v>
       </c>
       <c r="B50">
         <v>13</v>
@@ -3027,24 +2990,30 @@
         <v>49</v>
       </c>
       <c r="D50" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G50" s="1">
         <v>38327</v>
       </c>
       <c r="I50" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J50" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="K50" t="s">
+        <v>253</v>
       </c>
       <c r="M50" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.45">
+        <v>221</v>
+      </c>
+      <c r="P50" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B51">
         <v>14</v>
@@ -3053,24 +3022,30 @@
         <v>50</v>
       </c>
       <c r="D51" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="G51" s="1">
         <v>38776</v>
       </c>
       <c r="I51" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J51" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="K51" t="s">
+        <v>254</v>
       </c>
       <c r="M51" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.45">
+        <v>224</v>
+      </c>
+      <c r="P51" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B52">
         <v>16</v>
@@ -3079,24 +3054,30 @@
         <v>51</v>
       </c>
       <c r="D52" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="G52" s="1">
         <v>40848</v>
       </c>
       <c r="I52" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J52" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="K52" t="s">
+        <v>255</v>
       </c>
       <c r="M52" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.45">
+        <v>227</v>
+      </c>
+      <c r="P52" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B53">
         <v>33</v>
@@ -3105,26 +3086,33 @@
         <v>52</v>
       </c>
       <c r="D53" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="G53" s="1">
         <v>45223</v>
       </c>
       <c r="I53" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J53" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="K53" t="s">
+        <v>256</v>
       </c>
       <c r="M53" t="s">
-        <v>233</v>
+        <v>230</v>
+      </c>
+      <c r="P53" t="s">
+        <v>249</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="N16" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="P44" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="O44" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="K2" r:id="rId3" display="https://covers.openlibrary.org/b/id/10721368-M.jpg" xr:uid="{223B0864-F33B-4A9F-97F3-B9686705CAFD}"/>
+    <hyperlink ref="K37" r:id="rId4" xr:uid="{C5CFC9BF-F7AF-4A0F-AFAD-500592B4783E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>